<commit_message>
Use AnyaFinn as the dummy retailer in example data
AnyaFinn is Amplience's standard fictional retailer. Rebrands the example
workbook, CSVs, and docs accordingly.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/ecommerce-examples.xlsx
+++ b/examples/ecommerce-examples.xlsx
@@ -482,7 +482,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>HP-1001</t>
+          <t>AF-1001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -507,7 +507,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Harbour &amp; Pine</t>
+          <t>AnyaFinn</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -537,7 +537,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HP-1002</t>
+          <t>AF-1002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -562,7 +562,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Harbour &amp; Pine</t>
+          <t>AnyaFinn</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -592,7 +592,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HP-1003</t>
+          <t>AF-1003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Northwind</t>
+          <t>AnyaFinn</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HP-1004</t>
+          <t>AF-1004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Northwind</t>
+          <t>AnyaFinn</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -702,7 +702,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HP-1005</t>
+          <t>AF-1005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Harbour &amp; Pine</t>
+          <t>AnyaFinn</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -757,7 +757,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HP-1006</t>
+          <t>AF-1006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -782,7 +782,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Trailhead</t>
+          <t>AnyaFinn Active</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -812,7 +812,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HP-1007</t>
+          <t>AF-1007</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -837,7 +837,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Northwind</t>
+          <t>AnyaFinn</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -867,7 +867,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HP-1008</t>
+          <t>AF-1008</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -892,7 +892,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Harbour &amp; Pine</t>
+          <t>AnyaFinn Edit</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -922,7 +922,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HP-1009</t>
+          <t>AF-1009</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Harbour &amp; Pine</t>
+          <t>AnyaFinn</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HP-1010</t>
+          <t>AF-1010</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Trailhead</t>
+          <t>AnyaFinn Active</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1032,7 +1032,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>HP-1011</t>
+          <t>AF-1011</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Trailhead</t>
+          <t>AnyaFinn</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1087,7 +1087,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>HP-1012</t>
+          <t>AF-1012</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Harbour &amp; Pine</t>
+          <t>AnyaFinn Active</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2056,7 +2056,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Only for the Signature range</t>
+          <t>Only for the AnyaFinn Edit range</t>
         </is>
       </c>
     </row>

</xml_diff>